<commit_message>
DOC-001: plan German and English in backlog
U017 and T-U017-01..03 become Kern with the DE/EN decision noted. New
rows T-U017-04 (prepare English versions for review) and DOC-001, with
matching briefing rows; table ranges grow to A3:T141 and A3:G141.

Counting formulas no longer stop at row 139: Start C4 counts task ids,
C5/C6/C18 and Userstories J4:J36 count to row 1000 and ignore empty
rows via Tasks!$A$4:$A$1000<>"". Data validations extended the same
way. Start no longer carries a hardcoded task count, and the status
rule points at the Tasks sheet instead of GitHub Issues.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/VitaSync_Coding_Backlog.xlsx
+++ b/planning/VitaSync_Coding_Backlog.xlsx
@@ -344,8 +344,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TasksTable" displayName="TasksTable" ref="A3:T139" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A3:T139"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TasksTable" displayName="TasksTable" ref="A3:T141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A3:T141"/>
   <tableColumns count="20">
     <tableColumn id="1" name="Task-ID"/>
     <tableColumn id="2" name="Story-ID"/>
@@ -372,8 +372,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BriefingsTable" displayName="BriefingsTable" ref="A3:G139" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A3:G139"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BriefingsTable" displayName="BriefingsTable" ref="A3:G141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A3:G141"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Task-ID"/>
     <tableColumn id="2" name="Konkreter Auftrag"/>
@@ -637,10 +637,13 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>33 User Stories (U001–U033) und 136 Tasks einschließlich 18 Grundlagen. Nach D08 (kein Medizinprodukt) sind 4 Stories mit 13 Tasks gestrichen und weitere umgebaut; nach D09 (EU-Datenschutz, AI Act) kamen F016–F018, T-U028-03 und U033 hinzu. Siehe Spalten „Zweckprüfung (D08)“ und „Änderung“.</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="n"/>
+          <t>User Stories U001–U033 und die in der Spalte Anzahl gezaehlten Tasks, einschliesslich 18 Grundlagen. Nach D08 (kein Medizinprodukt) sind 4 Stories mit 13 Tasks gestrichen und weitere umgebaut; nach D09 (EU-Datenschutz, AI Act) kamen F016–F018, T-U028-03 und U033 hinzu. Siehe Spalten „Zweckprüfung (D08)“ und „Änderung“.</t>
+        </is>
+      </c>
+      <c r="C4" s="15">
+        <f>COUNTIFS(Tasks!$A$4:$A$1000,"&lt;&gt;")</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="67.5" customHeight="1" s="11">
       <c r="A5" s="16" t="inlineStr">
@@ -650,7 +653,7 @@
       </c>
       <c r="B5" s="16" t="n"/>
       <c r="C5" s="16">
-        <f>COUNTIFS(Tasks!$M$4:$M$139,"&lt;&gt;Erledigt",Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$M$4:$M$1000,"&lt;&gt;Erledigt",Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen",Tasks!$A$4:$A$1000,"&lt;&gt;")</f>
         <v/>
       </c>
     </row>
@@ -662,7 +665,7 @@
       </c>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="15">
-        <f>COUNTIFS(Tasks!$M$4:$M$139,"Erledigt")</f>
+        <f>COUNTIFS(Tasks!$M$4:$M$1000,"Erledigt")</f>
         <v/>
       </c>
     </row>
@@ -739,7 +742,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Ein Bearbeiter pro Task. Nach Implementierung: Im Review. Eine andere Person prüft und integriert. Erst dann Erledigt. Status und Zuweisung laufen über GitHub Issues (docs/Arbeitsablauf.md); diese Datei ist der Plan.</t>
+          <t>Ein Bearbeiter pro Task. Nach Implementierung: Im Review. Eine andere Person prüft und integriert; im Testlauf (D10) übernimmt eine Person alle Rollen und das Review ist die eigene Durchsicht des Diffs vor dem Merge. Erst dann Erledigt. Statusquelle ist die Spalte Status im Blatt Tasks; der Pull Request ist der Nachweis, in dem die Zeile im selben Zug gepflegt wird (docs/Arbeitsablauf.md). GitHub Issues sind optional.</t>
         </is>
       </c>
       <c r="C12" s="15" t="n"/>
@@ -817,7 +820,7 @@
       </c>
       <c r="B18" s="15" t="n"/>
       <c r="C18" s="15">
-        <f>COUNTIFS(Tasks!$M$4:$M$139,"Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$M$4:$M$1000,"Gestrichen")</f>
         <v/>
       </c>
     </row>
@@ -992,7 +995,7 @@
         </is>
       </c>
       <c r="J4" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A4,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A4,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K4" s="15" t="inlineStr">
@@ -1051,7 +1054,7 @@
         </is>
       </c>
       <c r="J5" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A5,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A5,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K5" s="16" t="inlineStr">
@@ -1110,7 +1113,7 @@
         </is>
       </c>
       <c r="J6" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A6,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A6,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K6" s="15" t="inlineStr">
@@ -1169,7 +1172,7 @@
         </is>
       </c>
       <c r="J7" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A7,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A7,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K7" s="16" t="inlineStr">
@@ -1224,7 +1227,7 @@
         </is>
       </c>
       <c r="J8" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A8,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A8,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K8" s="15" t="inlineStr">
@@ -1279,7 +1282,7 @@
         </is>
       </c>
       <c r="J9" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A9,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A9,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K9" s="16" t="inlineStr">
@@ -1338,7 +1341,7 @@
         </is>
       </c>
       <c r="J10" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A10,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A10,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K10" s="15" t="inlineStr">
@@ -1393,7 +1396,7 @@
         </is>
       </c>
       <c r="J11" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A11,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A11,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K11" s="16" t="inlineStr">
@@ -1452,7 +1455,7 @@
         </is>
       </c>
       <c r="J12" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A12,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A12,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K12" s="15" t="inlineStr">
@@ -1507,7 +1510,7 @@
         </is>
       </c>
       <c r="J13" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A13,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A13,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K13" s="16" t="inlineStr">
@@ -1562,7 +1565,7 @@
         </is>
       </c>
       <c r="J14" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A14,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A14,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K14" s="15" t="inlineStr">
@@ -1617,7 +1620,7 @@
         </is>
       </c>
       <c r="J15" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A15,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A15,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K15" s="16" t="inlineStr">
@@ -1672,7 +1675,7 @@
         </is>
       </c>
       <c r="J16" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A16,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A16,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K16" s="15" t="inlineStr">
@@ -1731,7 +1734,7 @@
         </is>
       </c>
       <c r="J17" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A17,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A17,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K17" s="16" t="inlineStr">
@@ -1790,7 +1793,7 @@
         </is>
       </c>
       <c r="J18" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A18,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A18,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K18" s="15" t="inlineStr">
@@ -1845,7 +1848,7 @@
         </is>
       </c>
       <c r="J19" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A19,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A19,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K19" s="16" t="inlineStr">
@@ -1896,11 +1899,11 @@
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Kern</t>
         </is>
       </c>
       <c r="J20" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A20,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A20,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K20" s="15" t="inlineStr">
@@ -1913,7 +1916,11 @@
           <t>Erlaubt</t>
         </is>
       </c>
-      <c r="M20" s="15" t="n"/>
+      <c r="M20" s="15" t="inlineStr">
+        <is>
+          <t>Entscheidung DE/EN 14.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="109.5" customHeight="1" s="11">
       <c r="A21" s="16" t="inlineStr">
@@ -1955,7 +1962,7 @@
         </is>
       </c>
       <c r="J21" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A21,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A21,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K21" s="16" t="inlineStr">
@@ -2014,7 +2021,7 @@
         </is>
       </c>
       <c r="J22" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A22,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A22,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K22" s="15" t="inlineStr">
@@ -2073,7 +2080,7 @@
         </is>
       </c>
       <c r="J23" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A23,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A23,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K23" s="16" t="inlineStr">
@@ -2128,7 +2135,7 @@
         </is>
       </c>
       <c r="J24" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A24,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A24,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K24" s="15" t="inlineStr">
@@ -2183,7 +2190,7 @@
         </is>
       </c>
       <c r="J25" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A25,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A25,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K25" s="16" t="inlineStr">
@@ -2238,7 +2245,7 @@
         </is>
       </c>
       <c r="J26" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A26,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A26,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K26" s="15" t="inlineStr">
@@ -2293,7 +2300,7 @@
         </is>
       </c>
       <c r="J27" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A27,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A27,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K27" s="16" t="inlineStr">
@@ -2348,7 +2355,7 @@
         </is>
       </c>
       <c r="J28" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A28,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A28,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K28" s="15" t="inlineStr">
@@ -2403,7 +2410,7 @@
         </is>
       </c>
       <c r="J29" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A29,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A29,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K29" s="16" t="inlineStr">
@@ -2458,7 +2465,7 @@
         </is>
       </c>
       <c r="J30" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A30,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A30,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K30" s="15" t="inlineStr">
@@ -2513,7 +2520,7 @@
         </is>
       </c>
       <c r="J31" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A31,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A31,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K31" s="16" t="inlineStr">
@@ -2568,7 +2575,7 @@
         </is>
       </c>
       <c r="J32" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A32,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A32,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K32" s="15" t="inlineStr">
@@ -2627,7 +2634,7 @@
         </is>
       </c>
       <c r="J33" s="16">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A33,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A33,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K33" s="16" t="inlineStr">
@@ -2686,7 +2693,7 @@
         </is>
       </c>
       <c r="J34" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A34,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A34,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K34" s="15" t="inlineStr">
@@ -2745,7 +2752,7 @@
         </is>
       </c>
       <c r="J35" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A35,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A35,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K35" s="15" t="inlineStr">
@@ -2804,7 +2811,7 @@
         </is>
       </c>
       <c r="J36" s="15">
-        <f>COUNTIFS(Tasks!$B$4:$B$139,A36,Tasks!$M$4:$M$139,"&lt;&gt;Gestrichen")</f>
+        <f>COUNTIFS(Tasks!$B$4:$B$1000,A36,Tasks!$M$4:$M$1000,"&lt;&gt;Gestrichen")</f>
         <v/>
       </c>
       <c r="K36" s="15" t="inlineStr">
@@ -2843,7 +2850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T139"/>
+  <dimension ref="A1:T141"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="10" min="1" max="1"/>
@@ -5393,7 +5400,7 @@
       </c>
       <c r="Q34" s="15" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Kern</t>
         </is>
       </c>
       <c r="R34" s="15" t="inlineStr">
@@ -5406,7 +5413,11 @@
           <t>Erlaubt</t>
         </is>
       </c>
-      <c r="T34" s="15" t="n"/>
+      <c r="T34" s="15" t="inlineStr">
+        <is>
+          <t>Entscheidung DE/EN 14.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="67.5" customHeight="1" s="11">
       <c r="A35" s="16" t="inlineStr">
@@ -5470,7 +5481,7 @@
       </c>
       <c r="Q35" s="16" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Kern</t>
         </is>
       </c>
       <c r="R35" s="16" t="inlineStr">
@@ -5483,7 +5494,11 @@
           <t>Erlaubt</t>
         </is>
       </c>
-      <c r="T35" s="16" t="n"/>
+      <c r="T35" s="16" t="inlineStr">
+        <is>
+          <t>Entscheidung DE/EN 14.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="67.5" customHeight="1" s="11">
       <c r="A36" s="15" t="inlineStr">
@@ -5547,7 +5562,7 @@
       </c>
       <c r="Q36" s="15" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Kern</t>
         </is>
       </c>
       <c r="R36" s="15" t="inlineStr">
@@ -5560,7 +5575,11 @@
           <t>Erlaubt</t>
         </is>
       </c>
-      <c r="T36" s="15" t="n"/>
+      <c r="T36" s="15" t="inlineStr">
+        <is>
+          <t>Entscheidung DE/EN 14.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="67.5" customHeight="1" s="11">
       <c r="A37" s="16" t="inlineStr">
@@ -13794,6 +13813,160 @@
       <c r="T139" s="15" t="inlineStr">
         <is>
           <t>Neu nach D09 (EU-Datenschutz/AI Act).</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="15" customHeight="1" s="11">
+      <c r="A140" s="15" t="inlineStr">
+        <is>
+          <t>T-U017-04</t>
+        </is>
+      </c>
+      <c r="B140" s="15" t="inlineStr">
+        <is>
+          <t>U017</t>
+        </is>
+      </c>
+      <c r="C140" s="15" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="D140" s="15" t="n"/>
+      <c r="E140" s="15" t="inlineStr">
+        <is>
+          <t>Englische Fassungen der Fachinhalte zur Prüfung vorbereiten</t>
+        </is>
+      </c>
+      <c r="F140" s="15" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="G140" s="19" t="n"/>
+      <c r="H140" s="19" t="n"/>
+      <c r="I140" s="18">
+        <f>(G140+H140)/2</f>
+        <v/>
+      </c>
+      <c r="J140" s="19" t="n"/>
+      <c r="K140" s="15" t="inlineStr">
+        <is>
+          <t>T-U009-01, T-U001-01</t>
+        </is>
+      </c>
+      <c r="L140" s="15" t="inlineStr">
+        <is>
+          <t>D07</t>
+        </is>
+      </c>
+      <c r="M140" s="19" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="N140" s="19" t="n"/>
+      <c r="O140" s="19" t="n"/>
+      <c r="P140" s="15" t="inlineStr">
+        <is>
+          <t>Unterstützend</t>
+        </is>
+      </c>
+      <c r="Q140" s="15" t="inlineStr">
+        <is>
+          <t>Kern</t>
+        </is>
+      </c>
+      <c r="R140" s="15" t="inlineStr">
+        <is>
+          <t>knowledge</t>
+        </is>
+      </c>
+      <c r="S140" s="15" t="inlineStr">
+        <is>
+          <t>Erlaubt</t>
+        </is>
+      </c>
+      <c r="T140" s="15" t="inlineStr">
+        <is>
+          <t>Neu nach Entscheidung DE/EN 14.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="15" customHeight="1" s="11">
+      <c r="A141" s="15" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="B141" s="15" t="inlineStr">
+        <is>
+          <t>BASIS</t>
+        </is>
+      </c>
+      <c r="C141" s="15" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="D141" s="15" t="n"/>
+      <c r="E141" s="15" t="inlineStr">
+        <is>
+          <t>Regelkonsistenz, knowledge-Format, Mehrsprachigkeit, Testlauf</t>
+        </is>
+      </c>
+      <c r="F141" s="15" t="inlineStr">
+        <is>
+          <t>Doku</t>
+        </is>
+      </c>
+      <c r="G141" s="19" t="n"/>
+      <c r="H141" s="19" t="n"/>
+      <c r="I141" s="18">
+        <f>(G141+H141)/2</f>
+        <v/>
+      </c>
+      <c r="J141" s="19" t="n"/>
+      <c r="K141" s="15" t="inlineStr">
+        <is>
+          <t>TEST-001, F002, F003</t>
+        </is>
+      </c>
+      <c r="L141" s="15" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="M141" s="19" t="inlineStr">
+        <is>
+          <t>Im Review</t>
+        </is>
+      </c>
+      <c r="N141" s="19" t="n"/>
+      <c r="O141" s="19" t="n"/>
+      <c r="P141" s="15" t="inlineStr">
+        <is>
+          <t>Nach menschlicher Freigabe</t>
+        </is>
+      </c>
+      <c r="Q141" s="15" t="inlineStr">
+        <is>
+          <t>Kern</t>
+        </is>
+      </c>
+      <c r="R141" s="15" t="inlineStr">
+        <is>
+          <t>docs, knowledge, contracts, scripts</t>
+        </is>
+      </c>
+      <c r="S141" s="15" t="inlineStr">
+        <is>
+          <t>Erlaubt</t>
+        </is>
+      </c>
+      <c r="T141" s="15" t="inlineStr">
+        <is>
+          <t>Neu nach TEST-001 und Entscheidungen 14.10.2026</t>
         </is>
       </c>
     </row>
@@ -13808,19 +13981,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="M4:M139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="M4:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
       <formula1>"Offen,Bereit,In Bearbeitung,Blockiert,Im Review,Erledigt,Gestrichen"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="O4:O139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="O4:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
       <formula1>"Mensch,Claude,Codex"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="G4:H139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="G4:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="J4:J139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="J4:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
       <formula1>"1,2,3,5"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -13840,7 +14013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G139"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="10" min="1" max="1"/>
@@ -18932,6 +19105,80 @@
       <c r="G139" s="15" t="inlineStr">
         <is>
           <t>U033</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="39.55" customHeight="1" s="11">
+      <c r="A140" s="15" t="inlineStr">
+        <is>
+          <t>T-U017-04</t>
+        </is>
+      </c>
+      <c r="B140" s="15" t="inlineStr">
+        <is>
+          <t>Bereite die englischen Fassungen der freigegebenen Fachinhalte zur fachlichen Prüfung vor. Gleiche id wie die deutsche Fassung, sprache en, Dateiname &lt;name&gt;.en.md.</t>
+        </is>
+      </c>
+      <c r="C140" s="15" t="inlineStr">
+        <is>
+          <t>Geprueft deutsche Fassung -&gt; englischer Entwurf zur Prüfung.</t>
+        </is>
+      </c>
+      <c r="D140" s="15" t="inlineStr">
+        <is>
+          <t>Je Inhalt existiert eine englische Datei mit gleicher id; Status hoechstens testfreigabe; kein Inhalt ohne deutsche Vorlage.</t>
+        </is>
+      </c>
+      <c r="E140" s="15" t="inlineStr">
+        <is>
+          <t>Fehlende englische Fassung führt zur deutschen Fassung mit Hinweis, nicht zu einer Übersetzung.</t>
+        </is>
+      </c>
+      <c r="F140" s="15" t="inlineStr">
+        <is>
+          <t>Nur den beschriebenen Teil umsetzen. Keine echten personenbezogenen Daten. Keine individuelle Bewertung, Diagnose oder Dringlichkeitseinstufung (D08). Keine maschinelle Übersetzung zur Laufzeit (harte Regel 12). Keine fachliche Freigabe setzen.</t>
+        </is>
+      </c>
+      <c r="G140" s="15" t="inlineStr">
+        <is>
+          <t>U017, D07</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="39.55" customHeight="1" s="11">
+      <c r="A141" s="15" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="B141" s="15" t="inlineStr">
+        <is>
+          <t>Siehe planning/work-orders/DOC-001.md.</t>
+        </is>
+      </c>
+      <c r="C141" s="15" t="inlineStr">
+        <is>
+          <t>Befunde aus TEST-001 und Entscheidungen vom 14.10.2026 -&gt; angepasste Regeln und Doku.</t>
+        </is>
+      </c>
+      <c r="D141" s="15" t="inlineStr">
+        <is>
+          <t>Siehe Arbeitsauftrag.</t>
+        </is>
+      </c>
+      <c r="E141" s="15" t="inlineStr">
+        <is>
+          <t>Strukturcheck im Gut- und Fehlerfall; Vertragsbeispiele inklusive Gegenprobe.</t>
+        </is>
+      </c>
+      <c r="F141" s="15" t="inlineStr">
+        <is>
+          <t>Nur den beschriebenen Teil umsetzen. Keine echten personenbezogenen Daten. Keine individuelle Bewertung, Diagnose oder Dringlichkeitseinstufung (D08). Kein Produktcode.</t>
+        </is>
+      </c>
+      <c r="G141" s="15" t="inlineStr">
+        <is>
+          <t>TEST-001, F002, F003</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DOC-001: sync task status after F002/F003 merge
F001 gets its owner, F002 and F003 move to Erledigt with the merged PR
noted. Handoffs record the merge and that the review was a single-person
diff review under D10; F003 work order names its reviewer.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/VitaSync_Coding_Backlog.xlsx
+++ b/planning/VitaSync_Coding_Backlog.xlsx
@@ -3041,8 +3041,16 @@
           <t>Erledigt</t>
         </is>
       </c>
-      <c r="N4" s="19" t="n"/>
-      <c r="O4" s="19" t="n"/>
+      <c r="N4" s="19" t="inlineStr">
+        <is>
+          <t>Atakan</t>
+        </is>
+      </c>
+      <c r="O4" s="19" t="inlineStr">
+        <is>
+          <t>Mensch</t>
+        </is>
+      </c>
       <c r="P4" s="15" t="inlineStr">
         <is>
           <t>Unterstützend</t>
@@ -3115,7 +3123,7 @@
       <c r="L5" s="16" t="n"/>
       <c r="M5" s="19" t="inlineStr">
         <is>
-          <t>Im Review</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="N5" s="19" t="inlineStr">
@@ -3148,7 +3156,11 @@
           <t>Erlaubt</t>
         </is>
       </c>
-      <c r="T5" s="16" t="n"/>
+      <c r="T5" s="16" t="inlineStr">
+        <is>
+          <t>PR #1 gemergt 14.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="67.5" customHeight="1" s="11">
       <c r="A6" s="15" t="inlineStr">
@@ -3200,11 +3212,19 @@
       <c r="L6" s="15" t="n"/>
       <c r="M6" s="19" t="inlineStr">
         <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="N6" s="19" t="n"/>
-      <c r="O6" s="19" t="n"/>
+          <t>Erledigt</t>
+        </is>
+      </c>
+      <c r="N6" s="19" t="inlineStr">
+        <is>
+          <t>Atakan</t>
+        </is>
+      </c>
+      <c r="O6" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
       <c r="P6" s="15" t="inlineStr">
         <is>
           <t>Unterstützend</t>
@@ -3225,7 +3245,11 @@
           <t>Erlaubt</t>
         </is>
       </c>
-      <c r="T6" s="15" t="n"/>
+      <c r="T6" s="15" t="inlineStr">
+        <is>
+          <t>PR #2 gemergt 14.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="67.5" customHeight="1" s="11">
       <c r="A7" s="16" t="inlineStr">

</xml_diff>

<commit_message>
DOC-001: mark task done after review
Relabel the Start counter in A5 from 'Offene Tasks' to 'Nicht erledigt'
because it also counts rows in review; the formula in C5 is unchanged.
DOC-001 moves to Erledigt with PR #3 noted.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/VitaSync_Coding_Backlog.xlsx
+++ b/planning/VitaSync_Coding_Backlog.xlsx
@@ -648,7 +648,7 @@
     <row r="5" ht="67.5" customHeight="1" s="11">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>Offene Tasks</t>
+          <t>Nicht erledigt</t>
         </is>
       </c>
       <c r="B5" s="16" t="n"/>
@@ -13963,7 +13963,7 @@
       </c>
       <c r="M141" s="19" t="inlineStr">
         <is>
-          <t>Im Review</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="N141" s="19" t="n"/>
@@ -13990,7 +13990,7 @@
       </c>
       <c r="T141" s="15" t="inlineStr">
         <is>
-          <t>Neu nach TEST-001 und Entscheidungen 14.10.2026</t>
+          <t>PR #3 gemergt 15.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F004: set own backlog row to in progress
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/VitaSync_Coding_Backlog.xlsx
+++ b/planning/VitaSync_Coding_Backlog.xlsx
@@ -3301,11 +3301,19 @@
       <c r="L7" s="16" t="n"/>
       <c r="M7" s="19" t="inlineStr">
         <is>
-          <t>Offen</t>
-        </is>
-      </c>
-      <c r="N7" s="19" t="n"/>
-      <c r="O7" s="19" t="n"/>
+          <t>In Bearbeitung</t>
+        </is>
+      </c>
+      <c r="N7" s="19" t="inlineStr">
+        <is>
+          <t>Atakan</t>
+        </is>
+      </c>
+      <c r="O7" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
       <c r="P7" s="16" t="inlineStr">
         <is>
           <t>Nach menschlicher Freigabe</t>

</xml_diff>

<commit_message>
F004: set own backlog row to in review
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/VitaSync_Coding_Backlog.xlsx
+++ b/planning/VitaSync_Coding_Backlog.xlsx
@@ -3301,7 +3301,7 @@
       <c r="L7" s="16" t="n"/>
       <c r="M7" s="19" t="inlineStr">
         <is>
-          <t>In Bearbeitung</t>
+          <t>Im Review</t>
         </is>
       </c>
       <c r="N7" s="19" t="inlineStr">
@@ -3334,7 +3334,11 @@
           <t>Erlaubt</t>
         </is>
       </c>
-      <c r="T7" s="16" t="n"/>
+      <c r="T7" s="16" t="inlineStr">
+        <is>
+          <t>PR #5, CI eingerichtet 15.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="67.5" customHeight="1" s="11">
       <c r="A8" s="15" t="inlineStr">

</xml_diff>

<commit_message>
F004: highlight finished tasks in the backlog
Conditional formatting instead of static fills, so a row turns green
when its status becomes Erledigt and loses the colour if that changes.
The existing Blockiert rule stopped at row 126 and now covers the same
range as the counting formulas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/VitaSync_Coding_Backlog.xlsx
+++ b/planning/VitaSync_Coding_Backlog.xlsx
@@ -196,7 +196,7 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -244,6 +244,17 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFF4DAD4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14011,9 +14022,14 @@
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
-  <conditionalFormatting sqref="M4:M126">
+  <conditionalFormatting sqref="M4:M1000">
     <cfRule type="containsText" rank="0" priority="2" equalAverage="0" operator="containsText" aboveAverage="0" dxfId="5" text="Blockiert" percent="0" bottom="0">
       <formula>NOT(ISERROR(SEARCH("Blockiert",M4)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:T1000">
+    <cfRule type="expression" priority="2" dxfId="6" stopIfTrue="0">
+      <formula>$M4="Erledigt"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">

</xml_diff>

<commit_message>
DOC-003: add work order, backlog row and handoff notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/VitaSync_Coding_Backlog.xlsx
+++ b/planning/VitaSync_Coding_Backlog.xlsx
@@ -344,7 +344,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TasksTable" displayName="TasksTable" ref="A3:T141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TasksTable" displayName="TasksTable" ref="A3:T142" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A3:T141"/>
   <tableColumns count="20">
     <tableColumn id="1" name="Task-ID"/>
@@ -372,7 +372,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BriefingsTable" displayName="BriefingsTable" ref="A3:G141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BriefingsTable" displayName="BriefingsTable" ref="A3:G142" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A3:G141"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Task-ID"/>
@@ -2850,7 +2850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T141"/>
+  <dimension ref="A1:T142"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="10" min="1" max="1"/>
@@ -13991,6 +13991,87 @@
       <c r="T141" s="15" t="inlineStr">
         <is>
           <t>PR #3 gemergt 15.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="15" customHeight="1" s="11">
+      <c r="A142" s="15" t="inlineStr">
+        <is>
+          <t>DOC-003</t>
+        </is>
+      </c>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>BASIS</t>
+        </is>
+      </c>
+      <c r="C142" s="15" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="D142" s="15" t="n"/>
+      <c r="E142" s="15" t="inlineStr">
+        <is>
+          <t>Abgleich Research gegen Regelwerk als Notiz</t>
+        </is>
+      </c>
+      <c r="F142" s="15" t="inlineStr">
+        <is>
+          <t>Doku</t>
+        </is>
+      </c>
+      <c r="G142" s="19" t="n"/>
+      <c r="H142" s="19" t="n"/>
+      <c r="I142" s="18">
+        <f>(G142+H142)/2</f>
+        <v/>
+      </c>
+      <c r="J142" s="19" t="n"/>
+      <c r="K142" s="15" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="L142" s="15" t="n"/>
+      <c r="M142" s="19" t="inlineStr">
+        <is>
+          <t>Im Review</t>
+        </is>
+      </c>
+      <c r="N142" s="19" t="inlineStr">
+        <is>
+          <t>Atakan</t>
+        </is>
+      </c>
+      <c r="O142" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="P142" s="15" t="inlineStr">
+        <is>
+          <t>Nach menschlicher Freigabe</t>
+        </is>
+      </c>
+      <c r="Q142" s="15" t="inlineStr">
+        <is>
+          <t>Kern</t>
+        </is>
+      </c>
+      <c r="R142" s="15" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="S142" s="15" t="inlineStr">
+        <is>
+          <t>Erlaubt</t>
+        </is>
+      </c>
+      <c r="T142" s="15" t="inlineStr">
+        <is>
+          <t>Notiz, keine Entscheidung; PR folgt</t>
         </is>
       </c>
     </row>
@@ -14037,7 +14118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="10" min="1" max="1"/>
@@ -19203,6 +19284,43 @@
       <c r="G141" s="15" t="inlineStr">
         <is>
           <t>TEST-001, F002, F003</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="39.55" customHeight="1" s="11">
+      <c r="A142" s="15" t="inlineStr">
+        <is>
+          <t>DOC-003</t>
+        </is>
+      </c>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>Siehe planning/work-orders/DOC-003.md.</t>
+        </is>
+      </c>
+      <c r="C142" s="15" t="inlineStr">
+        <is>
+          <t>research/ (10 Dateien) + Regelwerk -&gt; docs/Research-Abgleich.md.</t>
+        </is>
+      </c>
+      <c r="D142" s="15" t="inlineStr">
+        <is>
+          <t>Siehe Arbeitsauftrag.</t>
+        </is>
+      </c>
+      <c r="E142" s="15" t="inlineStr">
+        <is>
+          <t>Strukturcheck; Gegenlesen jeder Abweichung mit Quelle und Repo-Fundstelle.</t>
+        </is>
+      </c>
+      <c r="F142" s="15" t="inlineStr">
+        <is>
+          <t>Nur den beschriebenen Teil umsetzen. Keine Änderung an Entscheidungen, Regeln, contracts/ oder knowledge/. Keine neuen Backlog-Tasks. Keine individuelle Bewertung, Diagnose oder Dringlichkeitseinstufung (D08).</t>
+        </is>
+      </c>
+      <c r="G142" s="15" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DOC-004: add read-only rule, FHIR+OMOP and optional PHP/JS frontend
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/VitaSync_Coding_Backlog.xlsx
+++ b/planning/VitaSync_Coding_Backlog.xlsx
@@ -344,7 +344,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TasksTable" displayName="TasksTable" ref="A3:T141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TasksTable" displayName="TasksTable" ref="A3:T142" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A3:T141"/>
   <tableColumns count="20">
     <tableColumn id="1" name="Task-ID"/>
@@ -372,7 +372,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BriefingsTable" displayName="BriefingsTable" ref="A3:G141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BriefingsTable" displayName="BriefingsTable" ref="A3:G142" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A3:G141"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Task-ID"/>
@@ -2850,7 +2850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T141"/>
+  <dimension ref="A1:T1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="10" min="1" max="1"/>
@@ -13994,6 +13994,949 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="15" t="inlineStr">
+        <is>
+          <t>DOC-004</t>
+        </is>
+      </c>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>BASIS</t>
+        </is>
+      </c>
+      <c r="C142" s="15" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="D142" s="15" t="n"/>
+      <c r="E142" s="15" t="inlineStr">
+        <is>
+          <t>Regeln: Quelldaten nur lesen, FHIR und OMOP, optionales Frontend PHP/JS</t>
+        </is>
+      </c>
+      <c r="F142" s="15" t="inlineStr">
+        <is>
+          <t>Doku</t>
+        </is>
+      </c>
+      <c r="G142" s="19" t="n"/>
+      <c r="H142" s="19" t="n"/>
+      <c r="I142" s="18">
+        <f>(G142+H142)/2</f>
+        <v/>
+      </c>
+      <c r="J142" s="19" t="n"/>
+      <c r="K142" s="15" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="L142" s="15" t="inlineStr">
+        <is>
+          <t>D01, D02</t>
+        </is>
+      </c>
+      <c r="M142" s="19" t="inlineStr">
+        <is>
+          <t>Im Review</t>
+        </is>
+      </c>
+      <c r="N142" s="19" t="inlineStr">
+        <is>
+          <t>Atakan</t>
+        </is>
+      </c>
+      <c r="O142" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="P142" s="15" t="inlineStr">
+        <is>
+          <t>Nach menschlicher Freigabe</t>
+        </is>
+      </c>
+      <c r="Q142" s="15" t="inlineStr">
+        <is>
+          <t>Kern</t>
+        </is>
+      </c>
+      <c r="R142" s="15" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="S142" s="15" t="inlineStr">
+        <is>
+          <t>Erlaubt</t>
+        </is>
+      </c>
+      <c r="T142" s="15" t="inlineStr">
+        <is>
+          <t>Vorgaben Team 21.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
+    <row r="570"/>
+    <row r="571"/>
+    <row r="572"/>
+    <row r="573"/>
+    <row r="574"/>
+    <row r="575"/>
+    <row r="576"/>
+    <row r="577"/>
+    <row r="578"/>
+    <row r="579"/>
+    <row r="580"/>
+    <row r="581"/>
+    <row r="582"/>
+    <row r="583"/>
+    <row r="584"/>
+    <row r="585"/>
+    <row r="586"/>
+    <row r="587"/>
+    <row r="588"/>
+    <row r="589"/>
+    <row r="590"/>
+    <row r="591"/>
+    <row r="592"/>
+    <row r="593"/>
+    <row r="594"/>
+    <row r="595"/>
+    <row r="596"/>
+    <row r="597"/>
+    <row r="598"/>
+    <row r="599"/>
+    <row r="600"/>
+    <row r="601"/>
+    <row r="602"/>
+    <row r="603"/>
+    <row r="604"/>
+    <row r="605"/>
+    <row r="606"/>
+    <row r="607"/>
+    <row r="608"/>
+    <row r="609"/>
+    <row r="610"/>
+    <row r="611"/>
+    <row r="612"/>
+    <row r="613"/>
+    <row r="614"/>
+    <row r="615"/>
+    <row r="616"/>
+    <row r="617"/>
+    <row r="618"/>
+    <row r="619"/>
+    <row r="620"/>
+    <row r="621"/>
+    <row r="622"/>
+    <row r="623"/>
+    <row r="624"/>
+    <row r="625"/>
+    <row r="626"/>
+    <row r="627"/>
+    <row r="628"/>
+    <row r="629"/>
+    <row r="630"/>
+    <row r="631"/>
+    <row r="632"/>
+    <row r="633"/>
+    <row r="634"/>
+    <row r="635"/>
+    <row r="636"/>
+    <row r="637"/>
+    <row r="638"/>
+    <row r="639"/>
+    <row r="640"/>
+    <row r="641"/>
+    <row r="642"/>
+    <row r="643"/>
+    <row r="644"/>
+    <row r="645"/>
+    <row r="646"/>
+    <row r="647"/>
+    <row r="648"/>
+    <row r="649"/>
+    <row r="650"/>
+    <row r="651"/>
+    <row r="652"/>
+    <row r="653"/>
+    <row r="654"/>
+    <row r="655"/>
+    <row r="656"/>
+    <row r="657"/>
+    <row r="658"/>
+    <row r="659"/>
+    <row r="660"/>
+    <row r="661"/>
+    <row r="662"/>
+    <row r="663"/>
+    <row r="664"/>
+    <row r="665"/>
+    <row r="666"/>
+    <row r="667"/>
+    <row r="668"/>
+    <row r="669"/>
+    <row r="670"/>
+    <row r="671"/>
+    <row r="672"/>
+    <row r="673"/>
+    <row r="674"/>
+    <row r="675"/>
+    <row r="676"/>
+    <row r="677"/>
+    <row r="678"/>
+    <row r="679"/>
+    <row r="680"/>
+    <row r="681"/>
+    <row r="682"/>
+    <row r="683"/>
+    <row r="684"/>
+    <row r="685"/>
+    <row r="686"/>
+    <row r="687"/>
+    <row r="688"/>
+    <row r="689"/>
+    <row r="690"/>
+    <row r="691"/>
+    <row r="692"/>
+    <row r="693"/>
+    <row r="694"/>
+    <row r="695"/>
+    <row r="696"/>
+    <row r="697"/>
+    <row r="698"/>
+    <row r="699"/>
+    <row r="700"/>
+    <row r="701"/>
+    <row r="702"/>
+    <row r="703"/>
+    <row r="704"/>
+    <row r="705"/>
+    <row r="706"/>
+    <row r="707"/>
+    <row r="708"/>
+    <row r="709"/>
+    <row r="710"/>
+    <row r="711"/>
+    <row r="712"/>
+    <row r="713"/>
+    <row r="714"/>
+    <row r="715"/>
+    <row r="716"/>
+    <row r="717"/>
+    <row r="718"/>
+    <row r="719"/>
+    <row r="720"/>
+    <row r="721"/>
+    <row r="722"/>
+    <row r="723"/>
+    <row r="724"/>
+    <row r="725"/>
+    <row r="726"/>
+    <row r="727"/>
+    <row r="728"/>
+    <row r="729"/>
+    <row r="730"/>
+    <row r="731"/>
+    <row r="732"/>
+    <row r="733"/>
+    <row r="734"/>
+    <row r="735"/>
+    <row r="736"/>
+    <row r="737"/>
+    <row r="738"/>
+    <row r="739"/>
+    <row r="740"/>
+    <row r="741"/>
+    <row r="742"/>
+    <row r="743"/>
+    <row r="744"/>
+    <row r="745"/>
+    <row r="746"/>
+    <row r="747"/>
+    <row r="748"/>
+    <row r="749"/>
+    <row r="750"/>
+    <row r="751"/>
+    <row r="752"/>
+    <row r="753"/>
+    <row r="754"/>
+    <row r="755"/>
+    <row r="756"/>
+    <row r="757"/>
+    <row r="758"/>
+    <row r="759"/>
+    <row r="760"/>
+    <row r="761"/>
+    <row r="762"/>
+    <row r="763"/>
+    <row r="764"/>
+    <row r="765"/>
+    <row r="766"/>
+    <row r="767"/>
+    <row r="768"/>
+    <row r="769"/>
+    <row r="770"/>
+    <row r="771"/>
+    <row r="772"/>
+    <row r="773"/>
+    <row r="774"/>
+    <row r="775"/>
+    <row r="776"/>
+    <row r="777"/>
+    <row r="778"/>
+    <row r="779"/>
+    <row r="780"/>
+    <row r="781"/>
+    <row r="782"/>
+    <row r="783"/>
+    <row r="784"/>
+    <row r="785"/>
+    <row r="786"/>
+    <row r="787"/>
+    <row r="788"/>
+    <row r="789"/>
+    <row r="790"/>
+    <row r="791"/>
+    <row r="792"/>
+    <row r="793"/>
+    <row r="794"/>
+    <row r="795"/>
+    <row r="796"/>
+    <row r="797"/>
+    <row r="798"/>
+    <row r="799"/>
+    <row r="800"/>
+    <row r="801"/>
+    <row r="802"/>
+    <row r="803"/>
+    <row r="804"/>
+    <row r="805"/>
+    <row r="806"/>
+    <row r="807"/>
+    <row r="808"/>
+    <row r="809"/>
+    <row r="810"/>
+    <row r="811"/>
+    <row r="812"/>
+    <row r="813"/>
+    <row r="814"/>
+    <row r="815"/>
+    <row r="816"/>
+    <row r="817"/>
+    <row r="818"/>
+    <row r="819"/>
+    <row r="820"/>
+    <row r="821"/>
+    <row r="822"/>
+    <row r="823"/>
+    <row r="824"/>
+    <row r="825"/>
+    <row r="826"/>
+    <row r="827"/>
+    <row r="828"/>
+    <row r="829"/>
+    <row r="830"/>
+    <row r="831"/>
+    <row r="832"/>
+    <row r="833"/>
+    <row r="834"/>
+    <row r="835"/>
+    <row r="836"/>
+    <row r="837"/>
+    <row r="838"/>
+    <row r="839"/>
+    <row r="840"/>
+    <row r="841"/>
+    <row r="842"/>
+    <row r="843"/>
+    <row r="844"/>
+    <row r="845"/>
+    <row r="846"/>
+    <row r="847"/>
+    <row r="848"/>
+    <row r="849"/>
+    <row r="850"/>
+    <row r="851"/>
+    <row r="852"/>
+    <row r="853"/>
+    <row r="854"/>
+    <row r="855"/>
+    <row r="856"/>
+    <row r="857"/>
+    <row r="858"/>
+    <row r="859"/>
+    <row r="860"/>
+    <row r="861"/>
+    <row r="862"/>
+    <row r="863"/>
+    <row r="864"/>
+    <row r="865"/>
+    <row r="866"/>
+    <row r="867"/>
+    <row r="868"/>
+    <row r="869"/>
+    <row r="870"/>
+    <row r="871"/>
+    <row r="872"/>
+    <row r="873"/>
+    <row r="874"/>
+    <row r="875"/>
+    <row r="876"/>
+    <row r="877"/>
+    <row r="878"/>
+    <row r="879"/>
+    <row r="880"/>
+    <row r="881"/>
+    <row r="882"/>
+    <row r="883"/>
+    <row r="884"/>
+    <row r="885"/>
+    <row r="886"/>
+    <row r="887"/>
+    <row r="888"/>
+    <row r="889"/>
+    <row r="890"/>
+    <row r="891"/>
+    <row r="892"/>
+    <row r="893"/>
+    <row r="894"/>
+    <row r="895"/>
+    <row r="896"/>
+    <row r="897"/>
+    <row r="898"/>
+    <row r="899"/>
+    <row r="900"/>
+    <row r="901"/>
+    <row r="902"/>
+    <row r="903"/>
+    <row r="904"/>
+    <row r="905"/>
+    <row r="906"/>
+    <row r="907"/>
+    <row r="908"/>
+    <row r="909"/>
+    <row r="910"/>
+    <row r="911"/>
+    <row r="912"/>
+    <row r="913"/>
+    <row r="914"/>
+    <row r="915"/>
+    <row r="916"/>
+    <row r="917"/>
+    <row r="918"/>
+    <row r="919"/>
+    <row r="920"/>
+    <row r="921"/>
+    <row r="922"/>
+    <row r="923"/>
+    <row r="924"/>
+    <row r="925"/>
+    <row r="926"/>
+    <row r="927"/>
+    <row r="928"/>
+    <row r="929"/>
+    <row r="930"/>
+    <row r="931"/>
+    <row r="932"/>
+    <row r="933"/>
+    <row r="934"/>
+    <row r="935"/>
+    <row r="936"/>
+    <row r="937"/>
+    <row r="938"/>
+    <row r="939"/>
+    <row r="940"/>
+    <row r="941"/>
+    <row r="942"/>
+    <row r="943"/>
+    <row r="944"/>
+    <row r="945"/>
+    <row r="946"/>
+    <row r="947"/>
+    <row r="948"/>
+    <row r="949"/>
+    <row r="950"/>
+    <row r="951"/>
+    <row r="952"/>
+    <row r="953"/>
+    <row r="954"/>
+    <row r="955"/>
+    <row r="956"/>
+    <row r="957"/>
+    <row r="958"/>
+    <row r="959"/>
+    <row r="960"/>
+    <row r="961"/>
+    <row r="962"/>
+    <row r="963"/>
+    <row r="964"/>
+    <row r="965"/>
+    <row r="966"/>
+    <row r="967"/>
+    <row r="968"/>
+    <row r="969"/>
+    <row r="970"/>
+    <row r="971"/>
+    <row r="972"/>
+    <row r="973"/>
+    <row r="974"/>
+    <row r="975"/>
+    <row r="976"/>
+    <row r="977"/>
+    <row r="978"/>
+    <row r="979"/>
+    <row r="980"/>
+    <row r="981"/>
+    <row r="982"/>
+    <row r="983"/>
+    <row r="984"/>
+    <row r="985"/>
+    <row r="986"/>
+    <row r="987"/>
+    <row r="988"/>
+    <row r="989"/>
+    <row r="990"/>
+    <row r="991"/>
+    <row r="992"/>
+    <row r="993"/>
+    <row r="994"/>
+    <row r="995"/>
+    <row r="996"/>
+    <row r="997"/>
+    <row r="998"/>
+    <row r="999"/>
+    <row r="1000"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
@@ -14037,7 +14980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19" customWidth="1" style="10" min="1" max="1"/>
@@ -19203,6 +20146,43 @@
       <c r="G141" s="15" t="inlineStr">
         <is>
           <t>TEST-001, F002, F003</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="15" t="inlineStr">
+        <is>
+          <t>DOC-004</t>
+        </is>
+      </c>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>Siehe planning/work-orders/DOC-004.md.</t>
+        </is>
+      </c>
+      <c r="C142" s="15" t="inlineStr">
+        <is>
+          <t>Teamvorgaben -&gt; harte Regel 14, D01, D02, Architektur.</t>
+        </is>
+      </c>
+      <c r="D142" s="15" t="inlineStr">
+        <is>
+          <t>Siehe Arbeitsauftrag.</t>
+        </is>
+      </c>
+      <c r="E142" s="15" t="inlineStr">
+        <is>
+          <t>Strukturcheck.</t>
+        </is>
+      </c>
+      <c r="F142" s="15" t="inlineStr">
+        <is>
+          <t>Nur den beschriebenen Teil umsetzen. Kein Produktcode. Keine Änderung an D08. Keine individuelle Bewertung, Diagnose oder Dringlichkeitseinstufung (D08).</t>
+        </is>
+      </c>
+      <c r="G142" s="15" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
         </is>
       </c>
     </row>

</xml_diff>